<commit_message>
BIS-2791: Changed 'Type Group' into 'Type Groups' in XlsExport
</commit_message>
<xml_diff>
--- a/server-application-server/sourceTest/java/ch/ethz/sis/openbis/generic/server/xls/export/resources/export-sample-type-compatible-with-import.xlsx
+++ b/server-application-server/sourceTest/java/ch/ethz/sis/openbis/generic/server/xls/export/resources/export-sample-type-compatible-with-import.xlsx
@@ -52,7 +52,7 @@
     <t xml:space="preserve">Ontology Version</t>
   </si>
   <si>
-    <t xml:space="preserve">Type Group</t>
+    <t xml:space="preserve">Type Groups</t>
   </si>
   <si>
     <t xml:space="preserve">Meta Data</t>
@@ -155,7 +155,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -196,6 +196,28 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -241,7 +263,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -255,6 +277,22 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -275,8 +313,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S7"/>
-  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:S1048576"/>
+  <sheetFormatPr defaultColWidth="10.859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -318,7 +356,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
@@ -340,6 +378,7 @@
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
+      <c r="J3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
@@ -531,6 +570,28 @@
       <c r="R7" s="3"/>
       <c r="S7" s="3"/>
     </row>
+    <row r="9" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5"/>
+      <c r="C9" s="3"/>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="3"/>
+    </row>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>